<commit_message>
feat(menu): title screen, settings, pause and confirm UI
- TitleUI briefcase sheets (continue/new/settings) with raise-on-select TitleSheet
- TitleScene stops play time and opens the menu; continue loads latest save
- SettingsUI volumes and language, PauseUI with title confirm, generic ConfirmUI
- SaveSlotSelector (latest slot, new game slot, play time format) with tests
- Editor menu LOTW/UI/Build Title And Menus builds prefabs and Title scene (index 0)
- UIBuildUtil shared by notebook and menu builders; text keys for menus

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Table/Excel/Text.xlsx
+++ b/Table/Excel/Text.xlsx
@@ -125,8 +125,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TextTable" displayName="TextTable" ref="A1:D19" headerRowCount="1">
-  <autoFilter ref="A1:D19"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TextTable" displayName="TextTable" ref="A1:D39" headerRowCount="1">
+  <autoFilter ref="A1:D39"/>
   <tableColumns count="4">
     <tableColumn id="1" name="DataId"/>
     <tableColumn id="2" name="Key"/>
@@ -426,13 +426,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D19"/>
+  <dimension ref="A1:D39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
     <col width="27" customWidth="1" min="2" max="2"/>
-    <col width="28" customWidth="1" min="3" max="3"/>
-    <col width="32" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
+    <col width="58" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -814,6 +814,406 @@
       <c r="D19" t="inlineStr">
         <is>
           <t>Request done: {0}</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>113</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>ui.title.continue</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>이어하기</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Continue</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>114</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>ui.title.newgame</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>새로하기</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>New Game</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>115</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>ui.title.settings</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>설정</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Settings</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>116</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>ui.title.newgame.confirm</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>새로 시작하면 지금까지의 기록 위에 덮어씁니다. 시작할까요?</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Starting over will overwrite your record. Start?</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>117</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>ui.pause.header</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>잠시 멈춤</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Paused</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>118</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>ui.pause.resume</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>계속하기</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Resume</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>119</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>ui.pause.settings</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>설정</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Settings</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>120</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>ui.pause.title</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>타이틀로</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>To Title</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>121</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>ui.pause.title.confirm</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>마지막 저장 이후의 진행은 사라집니다. 타이틀로 갈까요?</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Progress since your last save will be lost. Go to title?</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>122</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>ui.settings.header</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>설정</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Settings</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>123</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>ui.settings.master</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>전체 음량</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Master</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>124</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>ui.settings.bgm</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>배경음</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Music</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>125</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>ui.settings.sfx</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>효과음</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Sound</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>126</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>ui.settings.language</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>언어</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Language</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>127</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>ui.language.name</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>한국어</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>128</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>ui.confirm.yes</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>예</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>129</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>ui.confirm.no</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>아니오</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>130</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>scene.Plaza</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>광장</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Plaza</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>131</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>scene.Character</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>테스트</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Test</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>132</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>ui.close</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>닫기</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Close</t>
         </is>
       </c>
     </row>

</xml_diff>